<commit_message>
auto(CY): 3h refresh 2026-05-14T19:35Z
</commit_message>
<xml_diff>
--- a/summary_2026-05-14.xlsx
+++ b/summary_2026-05-14.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CY — Party Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CY — Top by Spend" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CY — Top by Impressions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CY — Active Ads" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CY — Removed Ads" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MT — Party Overview" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MT — Active Ads" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="CY — Party Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CY — Top by Spend" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CY — Top by Impressions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CY — Active Ads" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CY — Removed Ads" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="MT — Party Overview" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="MT — Active Ads" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -611,10 +611,10 @@
         <v>312</v>
       </c>
       <c r="F5" t="n">
-        <v>808897</v>
+        <v>749900</v>
       </c>
       <c r="G5" t="n">
-        <v>10197</v>
+        <v>9900</v>
       </c>
     </row>
     <row r="6">
@@ -661,10 +661,10 @@
         <v>107</v>
       </c>
       <c r="F7" t="n">
-        <v>11998</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>198</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -861,10 +861,10 @@
         <v>18</v>
       </c>
       <c r="F15" t="n">
-        <v>479998</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>898</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -936,10 +936,10 @@
         <v>1537</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>1668856</v>
+        <v>1117863</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>14956</v>
+        <v>13563</v>
       </c>
     </row>
   </sheetData>
@@ -1066,13 +1066,13 @@
         <v>99</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>29999</v>
+        <v>24999</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>9009</v>
+        <v>8811</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>670909</v>
+        <v>620911</v>
       </c>
     </row>
     <row r="5">
@@ -1116,141 +1116,141 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Κληρίδης Αλέξανδρος</t>
+          <t>Ερωτοκρίτου Χριστιάνα</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>ΔΑ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Αλέξανδρος Κληρίδης / Alexandros Clerides</t>
+          <t>Χριστιάνα Ερωτοκρίτου</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>699</v>
+        <v>199</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>399999</v>
+        <v>89999</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>898</v>
+        <v>792</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>479998</v>
+        <v>90992</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ερωτοκρίτου Χριστιάνα</t>
+          <t>Φελλάς Μιχάλης</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Χριστιάνα Ερωτοκρίτου</t>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
         </is>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>75</v>
       </c>
       <c r="F7" t="n">
-        <v>17</v>
+        <v>71</v>
       </c>
       <c r="G7" t="n">
-        <v>199</v>
+        <v>499</v>
       </c>
       <c r="H7" t="n">
-        <v>89999</v>
+        <v>199999</v>
       </c>
       <c r="I7" t="n">
-        <v>792</v>
+        <v>693</v>
       </c>
       <c r="J7" t="n">
-        <v>90992</v>
+        <v>114993</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης</t>
+          <t>ΑΚΕΛ</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΑΚΕΛ</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+          <t>ΑΚΕΛ - AKEL</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>75</v>
+        <v>6</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>499</v>
+        <v>99</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>199999</v>
+        <v>24999</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>693</v>
+        <v>594</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>114993</v>
+        <v>49994</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ΑΚΕΛ</t>
+          <t>Πετρίδης Χαράλαμπος</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ΑΚΕΛ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ΑΚΕΛ - AKEL</t>
+          <t>Χαράλαμπος Πετρίδης - Charalambos Petrides</t>
         </is>
       </c>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="G9" t="n">
         <v>99</v>
@@ -1259,178 +1259,178 @@
         <v>24999</v>
       </c>
       <c r="I9" t="n">
-        <v>594</v>
+        <v>297</v>
       </c>
       <c r="J9" t="n">
-        <v>49994</v>
+        <v>35997</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Πετρίδης Χαράλαμπος</t>
+          <t>Θεμιστοκλέους Ανδρέας</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΔΕΚ</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Χαράλαμπος Πετρίδης - Charalambos Petrides</t>
+          <t>Ανδρέας Χρ. Θεμιστοκλέους</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>99</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>24999</v>
+        <v>5999</v>
       </c>
       <c r="I10" s="2" t="n">
         <v>297</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>35997</v>
+        <v>8997</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Θεμιστοκλέους Ανδρέας</t>
+          <t>Σαββίδης Χρύσανθος</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ΔΕΚ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Ανδρέας Χρ. Θεμιστοκλέους</t>
+          <t>Χρύσανθος Σαββίδης</t>
         </is>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G11" t="n">
-        <v>99</v>
+        <v>299</v>
       </c>
       <c r="H11" t="n">
-        <v>5999</v>
+        <v>149999</v>
       </c>
       <c r="I11" t="n">
-        <v>297</v>
+        <v>198</v>
       </c>
       <c r="J11" t="n">
-        <v>8997</v>
+        <v>33998</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Σαββίδης Χρύσανθος</t>
+          <t>Τσιρίδου Φωτεινή</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Χρύσανθος Σαββίδης</t>
+          <t>Φωτεινή Τσιρίδου - Fotini Tsiridou</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>299</v>
+        <v>99</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>149999</v>
+        <v>39999</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>198</v>
+        <v>99</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>33998</v>
+        <v>999</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Παλιος Νίκος</t>
+          <t>Σενέκης Χρίστος</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ΑΜΔΗ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Νίκος Παλιός</t>
+          <t>Χρίστος Σενέκης</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
         <v>99</v>
       </c>
       <c r="H13" t="n">
-        <v>14999</v>
+        <v>3999</v>
       </c>
       <c r="I13" t="n">
-        <v>198</v>
+        <v>99</v>
       </c>
       <c r="J13" t="n">
-        <v>11998</v>
+        <v>3999</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Τσιρίδου Φωτεινή</t>
+          <t>Νικολαΐδης Ζήνωνας</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΟΙΚΟΛΟΓΟΙ</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Φωτεινή Τσιρίδου - Fotini Tsiridou</t>
+          <t>Zenonas Nicolaides</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
@@ -1440,159 +1440,159 @@
         <v>1</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>99</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>39999</v>
+        <v>14999</v>
       </c>
       <c r="I14" s="2" t="n">
         <v>99</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>999</v>
+        <v>14999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Σενέκης Χρίστος</t>
+          <t>Μούντουκκος Κωνσταντίνος</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Χρίστος Σενέκης</t>
+          <t>Constantinos Mountouckos</t>
         </is>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G15" t="n">
         <v>99</v>
       </c>
       <c r="H15" t="n">
-        <v>3999</v>
+        <v>14999</v>
       </c>
       <c r="I15" t="n">
         <v>99</v>
       </c>
       <c r="J15" t="n">
-        <v>3999</v>
+        <v>14999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Παπαδοπουλος Γεώργιος</t>
+          <t>Χειμωνίδης Ανδρέας</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΑΛΜΑ</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Γεώργιος Παπαδόπουλος-Georgios Papadopoulos</t>
+          <t>Δρ Ανδρέας Χειμωνίδης - Υποψήφιος Βουλευτής Λεμεσού</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>99</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>8999</v>
+        <v>4999</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>8999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Νικολαΐδης Ζήνωνας</t>
+          <t>Χατζηπαυλου Αυγή</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ΟΙΚΟΛΟΓΟΙ</t>
+          <t>ΑΚΕΛ</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Zenonas Nicolaides</t>
+          <t>ΠΟΓΟ Λευκωσίας - Κερύνειας</t>
         </is>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>14999</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>14999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Μούντουκκος Κωνσταντίνος</t>
+          <t>Χαπεσιάν Άρι</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Constantinos Mountouckos</t>
+          <t>Ari Habeshian-Άρι Χαπεσιάν</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>99</v>
@@ -1601,42 +1601,42 @@
         <v>14999</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>14999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Χειμωνίδης Ανδρέας</t>
+          <t>Χαμπούλλας Ευγένιος</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ΑΛΜΑ</t>
+          <t>ΕΛΑΜ</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Δρ Ανδρέας Χειμωνίδης - Υποψήφιος Βουλευτής Λεμεσού</t>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G19" t="n">
         <v>99</v>
       </c>
       <c r="H19" t="n">
-        <v>4999</v>
+        <v>8999</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
@@ -1648,27 +1648,27 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Χατζηπαυλου Αυγή</t>
+          <t>Φράγκου Αντωνία</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>ΑΚΕΛ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>ΠΟΓΟ Λευκωσίας - Κερύνειας</t>
+          <t>antoniafrangou2026</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>0</v>
@@ -1686,33 +1686,33 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Χαπεσιάν Άρι</t>
+          <t>Φλουρεντζου Μάριος</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ΔΗΠΑ</t>
+          <t>ΕΛΑΜ</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ari Habeshian-Άρι Χαπεσιάν</t>
+          <t>Marios Flourentzou</t>
         </is>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="G21" t="n">
         <v>99</v>
       </c>
       <c r="H21" t="n">
-        <v>14999</v>
+        <v>5999</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -1724,7 +1724,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Χαμπούλλας Ευγένιος</t>
+          <t>Φλουρέντζου Μάριος</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1734,23 +1734,23 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+          <t>Μάριος Φλουρέντζου - Μαζί για την Αμμόχωστο</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E22" s="2" t="n">
-        <v>62</v>
-      </c>
       <c r="F22" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>8999</v>
+        <v>0</v>
       </c>
       <c r="I22" s="2" t="n">
         <v>0</v>
@@ -1762,33 +1762,33 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Φράγκου Αντωνία</t>
+          <t>Φελλας Μιχάλης</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>antoniafrangou2026</t>
+          <t>Michalis Fellas</t>
         </is>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>19999</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -1800,33 +1800,33 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Φλουρεντζου Μάριος</t>
+          <t>Τσολάκη Ευανθία</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>ΕΛΑΜ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Marios Flourentzou</t>
+          <t>Ευανθία - Εύη - Τσολάκη</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>99</v>
+        <v>299</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>5999</v>
+        <v>249999</v>
       </c>
       <c r="I24" s="2" t="n">
         <v>0</v>
@@ -1838,33 +1838,33 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Φλουρέντζου Μάριος</t>
+          <t>Τσατσου Θεόδωρος</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ΕΛΑΜ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Μάριος Φλουρέντζου - Μαζί για την Αμμόχωστο</t>
+          <t>Θεόδωρος Τσάτσου - Theodoros Tsatsou</t>
         </is>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>2999</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -1876,33 +1876,33 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Φελλας Μιχάλης</t>
+          <t>Τσαγγάρης Ανδρέας</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΣΗΚΟΥ ΠΑΝΩ</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Michalis Fellas</t>
+          <t>Αντρέας Τσαγγάρης - ΣΗΚΟΥ ΠΑΝΩ</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="2" t="n">
-        <v>20</v>
-      </c>
       <c r="F26" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>19999</v>
+        <v>0</v>
       </c>
       <c r="I26" s="2" t="n">
         <v>0</v>
@@ -1914,33 +1914,33 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Τσολάκη Ευανθία</t>
+          <t>Σωτηρίου Ανδρέας</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΕΚ</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ευανθία - Εύη - Τσολάκη</t>
+          <t>ΔΕΚ - Δημοκρατικό Εθνικό Κίνημα</t>
         </is>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>299</v>
+        <v>99</v>
       </c>
       <c r="H27" t="n">
-        <v>249999</v>
+        <v>5999</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -1952,24 +1952,24 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Τσατσου Θεόδωρος</t>
+          <t>Στυλιανού Στέλιος</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΕΝΕΡΓΟΙ ΠΟΛΙΤΕΣ</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Θεόδωρος Τσάτσου - Theodoros Tsatsou</t>
+          <t>Stelios Stylianou</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>1</v>
@@ -1978,7 +1978,7 @@
         <v>99</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>2999</v>
+        <v>8999</v>
       </c>
       <c r="I28" s="2" t="n">
         <v>0</v>
@@ -1990,24 +1990,24 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Τσαγγάρης Ανδρέας</t>
+          <t>Στυλιανού Μάριος</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ΣΗΚΟΥ ΠΑΝΩ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Αντρέας Τσαγγάρης - ΣΗΚΟΥ ΠΑΝΩ</t>
+          <t>olathrepivatis</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -2028,33 +2028,33 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Σωτηρίου Ανδρέας</t>
+          <t>Στυλιανού Μάριος</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>ΔΕΚ</t>
+          <t>ΑΛΜΑ</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>ΔΕΚ - Δημοκρατικό Εθνικό Κίνημα</t>
+          <t>Μάριος Στυλιανού</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>99</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>5999</v>
+        <v>4999</v>
       </c>
       <c r="I30" s="2" t="n">
         <v>0</v>
@@ -2066,33 +2066,33 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Στυλιανού Στέλιος</t>
+          <t>Στυλιανού Μάριος</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ΕΝΕΡΓΟΙ ΠΟΛΙΤΕΣ</t>
+          <t>ΑΚΕΛ</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Stelios Stylianou</t>
+          <t>Marios Stylianou</t>
         </is>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>8999</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
@@ -2104,33 +2104,33 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Στυλιανού Μάριος</t>
+          <t>Στυλιανού Γιώργος</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΠΑ</t>
+          <t>ΔΕΚ</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>olathrepivatis</t>
+          <t>Δημοκρατική Αλλαγή</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>0</v>
+        <v>3999</v>
       </c>
       <c r="I32" s="2" t="n">
         <v>0</v>
@@ -2142,33 +2142,33 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Στυλιανού Μάριος</t>
+          <t>Στυλιανού Γιάννος</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ΑΛΜΑ</t>
+          <t>ΕΔΕΚ</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Μάριος Στυλιανού</t>
+          <t>Στυλιανού Γιάννος</t>
         </is>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>4999</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
@@ -2301,191 +2301,191 @@
         <v>99</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>29999</v>
+        <v>24999</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>9009</v>
+        <v>8811</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>670909</v>
+        <v>620911</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Κληρίδης Αλέξανδρος</t>
+          <t>Παπαβασιλείου Σταμάτης</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ΔΑ</t>
+          <t>ΟΙΚΟΛΟΓΟΙ</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Αλέξανδρος Κληρίδης / Alexandros Clerides</t>
+          <t>Σταμάτης Στάμος Παπαβασιλείου</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G5" t="n">
-        <v>699</v>
+        <v>99</v>
       </c>
       <c r="H5" t="n">
-        <v>399999</v>
+        <v>19999</v>
       </c>
       <c r="I5" t="n">
-        <v>898</v>
+        <v>1485</v>
       </c>
       <c r="J5" t="n">
-        <v>479998</v>
+        <v>126985</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Παπαβασιλείου Σταμάτης</t>
+          <t>Φελλάς Μιχάλης</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>ΟΙΚΟΛΟΓΟΙ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Σταμάτης Στάμος Παπαβασιλείου</t>
+          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>99</v>
+        <v>499</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>19999</v>
+        <v>199999</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>1485</v>
+        <v>693</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>126985</v>
+        <v>114993</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης</t>
+          <t>Ερωτοκρίτου Χριστιάνα</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Φελλάς Μιχάλης Δημοτικός Σύμβουλος Λεμεσού</t>
+          <t>Χριστιάνα Ερωτοκρίτου</t>
         </is>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>75</v>
+        <v>8</v>
       </c>
       <c r="F7" t="n">
-        <v>71</v>
+        <v>17</v>
       </c>
       <c r="G7" t="n">
-        <v>499</v>
+        <v>199</v>
       </c>
       <c r="H7" t="n">
-        <v>199999</v>
+        <v>89999</v>
       </c>
       <c r="I7" t="n">
-        <v>693</v>
+        <v>792</v>
       </c>
       <c r="J7" t="n">
-        <v>114993</v>
+        <v>90992</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Ερωτοκρίτου Χριστιάνα</t>
+          <t>ΑΚΕΛ</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΑΚΕΛ</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Χριστιάνα Ερωτοκρίτου</t>
+          <t>ΑΚΕΛ - AKEL</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>199</v>
+        <v>99</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>89999</v>
+        <v>24999</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>792</v>
+        <v>594</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>90992</v>
+        <v>49994</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ΑΚΕΛ</t>
+          <t>Πετρίδης Χαράλαμπος</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ΑΚΕΛ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ΑΚΕΛ - AKEL</t>
+          <t>Χαράλαμπος Πετρίδης - Charalambos Petrides</t>
         </is>
       </c>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="G9" t="n">
         <v>99</v>
@@ -2494,112 +2494,112 @@
         <v>24999</v>
       </c>
       <c r="I9" t="n">
-        <v>594</v>
+        <v>297</v>
       </c>
       <c r="J9" t="n">
-        <v>49994</v>
+        <v>35997</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Πετρίδης Χαράλαμπος</t>
+          <t>Σαββίδης Χρύσανθος</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Χαράλαμπος Πετρίδης - Charalambos Petrides</t>
+          <t>Χρύσανθος Σαββίδης</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>99</v>
+        <v>299</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>24999</v>
+        <v>149999</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>297</v>
+        <v>198</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>35997</v>
+        <v>33998</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Σαββίδης Χρύσανθος</t>
+          <t>Νικολαΐδης Ζήνωνας</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΟΙΚΟΛΟΓΟΙ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Χρύσανθος Σαββίδης</t>
+          <t>Zenonas Nicolaides</t>
         </is>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>299</v>
+        <v>99</v>
       </c>
       <c r="H11" t="n">
-        <v>149999</v>
+        <v>14999</v>
       </c>
       <c r="I11" t="n">
-        <v>198</v>
+        <v>99</v>
       </c>
       <c r="J11" t="n">
-        <v>33998</v>
+        <v>14999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Νικολαΐδης Ζήνωνας</t>
+          <t>Μούντουκκος Κωνσταντίνος</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>ΟΙΚΟΛΟΓΟΙ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Zenonas Nicolaides</t>
+          <t>Constantinos Mountouckos</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>99</v>
@@ -2617,207 +2617,207 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Μούντουκκος Κωνσταντίνος</t>
+          <t>Θεμιστοκλέους Ανδρέας</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΔΕΚ</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Constantinos Mountouckos</t>
+          <t>Ανδρέας Χρ. Θεμιστοκλέους</t>
         </is>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G13" t="n">
         <v>99</v>
       </c>
       <c r="H13" t="n">
-        <v>14999</v>
+        <v>5999</v>
       </c>
       <c r="I13" t="n">
-        <v>99</v>
+        <v>297</v>
       </c>
       <c r="J13" t="n">
-        <v>14999</v>
+        <v>8997</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Παλιος Νίκος</t>
+          <t>Σενέκης Χρίστος</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>ΑΜΔΗ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Νίκος Παλιός</t>
+          <t>Χρίστος Σενέκης</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>99</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>14999</v>
+        <v>3999</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>198</v>
+        <v>99</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>11998</v>
+        <v>3999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Παπαδοπουλος Γεώργιος</t>
+          <t>Τσιρίδου Φωτεινή</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Γεώργιος Παπαδόπουλος-Georgios Papadopoulos</t>
+          <t>Φωτεινή Τσιρίδου - Fotini Tsiridou</t>
         </is>
       </c>
       <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
         <v>1</v>
       </c>
-      <c r="E15" t="n">
-        <v>4</v>
-      </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G15" t="n">
         <v>99</v>
       </c>
       <c r="H15" t="n">
-        <v>8999</v>
+        <v>39999</v>
       </c>
       <c r="I15" t="n">
         <v>99</v>
       </c>
       <c r="J15" t="n">
-        <v>8999</v>
+        <v>999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Θεμιστοκλέους Ανδρέας</t>
+          <t>Χειμωνίδης Ανδρέας</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>ΔΕΚ</t>
+          <t>ΑΛΜΑ</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Ανδρέας Χρ. Θεμιστοκλέους</t>
+          <t>Δρ Ανδρέας Χειμωνίδης - Υποψήφιος Βουλευτής Λεμεσού</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>99</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>5999</v>
+        <v>4999</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>297</v>
+        <v>0</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>8997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Σενέκης Χρίστος</t>
+          <t>Χατζηπαυλου Αυγή</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΑΚΕΛ</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Χρίστος Σενέκης</t>
+          <t>ΠΟΓΟ Λευκωσίας - Κερύνειας</t>
         </is>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>3999</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>3999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Τσιρίδου Φωτεινή</t>
+          <t>Χαπεσιάν Άρι</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Φωτεινή Τσιρίδου - Fotini Tsiridou</t>
+          <t>Ari Habeshian-Άρι Χαπεσιάν</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
@@ -2827,51 +2827,51 @@
         <v>1</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>99</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>39999</v>
+        <v>14999</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Χειμωνίδης Ανδρέας</t>
+          <t>Χαμπούλλας Ευγένιος</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ΑΛΜΑ</t>
+          <t>ΕΛΑΜ</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Δρ Ανδρέας Χειμωνίδης - Υποψήφιος Βουλευτής Λεμεσού</t>
+          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G19" t="n">
         <v>99</v>
       </c>
       <c r="H19" t="n">
-        <v>4999</v>
+        <v>8999</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
@@ -2883,27 +2883,27 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Χατζηπαυλου Αυγή</t>
+          <t>Φράγκου Αντωνία</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>ΑΚΕΛ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>ΠΟΓΟ Λευκωσίας - Κερύνειας</t>
+          <t>antoniafrangou2026</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>0</v>
@@ -2921,33 +2921,33 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Χαπεσιάν Άρι</t>
+          <t>Φλουρεντζου Μάριος</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ΔΗΠΑ</t>
+          <t>ΕΛΑΜ</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ari Habeshian-Άρι Χαπεσιάν</t>
+          <t>Marios Flourentzou</t>
         </is>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="G21" t="n">
         <v>99</v>
       </c>
       <c r="H21" t="n">
-        <v>14999</v>
+        <v>5999</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -2959,7 +2959,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Χαμπούλλας Ευγένιος</t>
+          <t>Φλουρέντζου Μάριος</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2969,23 +2969,23 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Evgenios Hamboullas | Ευγένιος Χαμπουλλάς</t>
+          <t>Μάριος Φλουρέντζου - Μαζί για την Αμμόχωστο</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E22" s="2" t="n">
-        <v>62</v>
-      </c>
       <c r="F22" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>8999</v>
+        <v>0</v>
       </c>
       <c r="I22" s="2" t="n">
         <v>0</v>
@@ -2997,33 +2997,33 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Φράγκου Αντωνία</t>
+          <t>Φελλας Μιχάλης</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>antoniafrangou2026</t>
+          <t>Michalis Fellas</t>
         </is>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>19999</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -3035,33 +3035,33 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Φλουρεντζου Μάριος</t>
+          <t>Τσολάκη Ευανθία</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>ΕΛΑΜ</t>
+          <t>ΔΗΚΟ</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Marios Flourentzou</t>
+          <t>Ευανθία - Εύη - Τσολάκη</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>99</v>
+        <v>299</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>5999</v>
+        <v>249999</v>
       </c>
       <c r="I24" s="2" t="n">
         <v>0</v>
@@ -3073,33 +3073,33 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Φλουρέντζου Μάριος</t>
+          <t>Τσατσου Θεόδωρος</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ΕΛΑΜ</t>
+          <t>ΔΗΣΥ</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Μάριος Φλουρέντζου - Μαζί για την Αμμόχωστο</t>
+          <t>Θεόδωρος Τσάτσου - Theodoros Tsatsou</t>
         </is>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>2999</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -3111,33 +3111,33 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Φελλας Μιχάλης</t>
+          <t>Τσαγγάρης Ανδρέας</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΣΗΚΟΥ ΠΑΝΩ</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Michalis Fellas</t>
+          <t>Αντρέας Τσαγγάρης - ΣΗΚΟΥ ΠΑΝΩ</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="2" t="n">
-        <v>20</v>
-      </c>
       <c r="F26" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>19999</v>
+        <v>0</v>
       </c>
       <c r="I26" s="2" t="n">
         <v>0</v>
@@ -3149,33 +3149,33 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Τσολάκη Ευανθία</t>
+          <t>Σωτηρίου Ανδρέας</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ΔΗΚΟ</t>
+          <t>ΔΕΚ</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ευανθία - Εύη - Τσολάκη</t>
+          <t>ΔΕΚ - Δημοκρατικό Εθνικό Κίνημα</t>
         </is>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>299</v>
+        <v>99</v>
       </c>
       <c r="H27" t="n">
-        <v>249999</v>
+        <v>5999</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -3187,24 +3187,24 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Τσατσου Θεόδωρος</t>
+          <t>Στυλιανού Στέλιος</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΣΥ</t>
+          <t>ΕΝΕΡΓΟΙ ΠΟΛΙΤΕΣ</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Θεόδωρος Τσάτσου - Theodoros Tsatsou</t>
+          <t>Stelios Stylianou</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>1</v>
@@ -3213,7 +3213,7 @@
         <v>99</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>2999</v>
+        <v>8999</v>
       </c>
       <c r="I28" s="2" t="n">
         <v>0</v>
@@ -3225,24 +3225,24 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Τσαγγάρης Ανδρέας</t>
+          <t>Στυλιανού Μάριος</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ΣΗΚΟΥ ΠΑΝΩ</t>
+          <t>ΔΗΠΑ</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Αντρέας Τσαγγάρης - ΣΗΚΟΥ ΠΑΝΩ</t>
+          <t>olathrepivatis</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
@@ -3263,33 +3263,33 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Σωτηρίου Ανδρέας</t>
+          <t>Στυλιανού Μάριος</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>ΔΕΚ</t>
+          <t>ΑΛΜΑ</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>ΔΕΚ - Δημοκρατικό Εθνικό Κίνημα</t>
+          <t>Μάριος Στυλιανού</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>99</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>5999</v>
+        <v>4999</v>
       </c>
       <c r="I30" s="2" t="n">
         <v>0</v>
@@ -3301,33 +3301,33 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Στυλιανού Στέλιος</t>
+          <t>Στυλιανού Μάριος</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ΕΝΕΡΓΟΙ ΠΟΛΙΤΕΣ</t>
+          <t>ΑΚΕΛ</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Stelios Stylianou</t>
+          <t>Marios Stylianou</t>
         </is>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>8999</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
@@ -3339,33 +3339,33 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Στυλιανού Μάριος</t>
+          <t>Στυλιανού Γιώργος</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>ΔΗΠΑ</t>
+          <t>ΔΕΚ</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>olathrepivatis</t>
+          <t>Δημοκρατική Αλλαγή</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>0</v>
+        <v>3999</v>
       </c>
       <c r="I32" s="2" t="n">
         <v>0</v>
@@ -3377,33 +3377,33 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Στυλιανού Μάριος</t>
+          <t>Στυλιανού Γιάννος</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ΑΛΜΑ</t>
+          <t>ΕΔΕΚ</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Μάριος Στυλιανού</t>
+          <t>Στυλιανού Γιάννος</t>
         </is>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>4999</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
@@ -3433,8 +3433,8 @@
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -3536,16 +3536,8 @@
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>15,000–19,999</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>0–99</t>
-        </is>
-      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3622,16 +3614,8 @@
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>25,000–29,999</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>0–99</t>
-        </is>
-      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3786,16 +3770,8 @@
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>3,000–3,999</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>0–99</t>
-        </is>
-      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3833,16 +3809,8 @@
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>7,000–7,999</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>0–99</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -4348,16 +4316,8 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>8,000–8,999</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>0–99</t>
-        </is>
-      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4434,16 +4394,8 @@
           <t>2026-03-28</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>350,000–399,999</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>600–699</t>
-        </is>
-      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4637,16 +4589,8 @@
           <t>2026-02-28</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>70,000–79,999</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>100–199</t>
-        </is>
-      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">

</xml_diff>